<commit_message>
Refine factory particle texture profile
</commit_message>
<xml_diff>
--- a/skills/magnetic-cube-scene-workflow/assets/dual_factory_library/workbooks/表格2.xlsx
+++ b/skills/magnetic-cube-scene-workflow/assets/dual_factory_library/workbooks/表格2.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="颗粒" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="颗粒" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'颗粒'!$A$1:$AG$20</definedName>
@@ -199,7 +199,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -214,13 +214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -239,13 +239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -264,13 +264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -289,13 +289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -314,13 +314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -339,13 +339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -364,13 +364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -389,13 +389,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId8"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -414,13 +414,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId9"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -439,13 +439,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId10"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId10"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -464,13 +464,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId11"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId11"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -489,13 +489,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId12"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -514,13 +514,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId13"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -539,13 +539,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId14"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -564,13 +564,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId15"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -589,13 +589,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -614,13 +614,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -639,13 +639,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId18"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -664,13 +664,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId19"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -689,13 +689,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId20"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -714,13 +714,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId21"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -739,13 +739,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId22"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -764,13 +764,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId23"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -789,13 +789,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId24"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -814,13 +814,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId25"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -839,13 +839,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId26"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -864,13 +864,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId27"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -889,13 +889,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId28"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -914,13 +914,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId29"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -939,13 +939,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId30"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -964,13 +964,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -989,13 +989,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId32"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1014,13 +1014,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId33"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1039,13 +1039,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId34"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1064,13 +1064,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId35"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1089,13 +1089,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId36"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1114,13 +1114,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId37"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1139,13 +1139,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId38"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1164,13 +1164,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId39"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1189,13 +1189,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId40"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId40"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1214,13 +1214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId41"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId41"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1239,13 +1239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId42"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId42"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1264,13 +1264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId43"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId43"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1289,13 +1289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId44"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId44"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1314,13 +1314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId45"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId45"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1339,13 +1339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId46"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId46"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1364,13 +1364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId47"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId47"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1389,13 +1389,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId48"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId48"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1414,13 +1414,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId49"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId49"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1439,13 +1439,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId50"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId50"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1464,13 +1464,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId51"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId51"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1489,13 +1489,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId52"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId52"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1514,13 +1514,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId53"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId53"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1539,13 +1539,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId54"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId54"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1564,13 +1564,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId55"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId55"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1589,13 +1589,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId56"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId56"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1614,13 +1614,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId57"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId57"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1639,13 +1639,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId58"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId58"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1664,13 +1664,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId59"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId59"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1689,13 +1689,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId60"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId60"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1714,13 +1714,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId61"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId61"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1739,13 +1739,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId62"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId62"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1764,13 +1764,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId63"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId63"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1789,13 +1789,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId64"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId64"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1814,13 +1814,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId65"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId65"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1839,13 +1839,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId66"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId66"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1864,13 +1864,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId67"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId67"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1889,13 +1889,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId68"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId68"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1914,13 +1914,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId69"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId69"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1939,13 +1939,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId70"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId70"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1964,13 +1964,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId71"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId71"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -1989,13 +1989,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId72"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId72"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2014,13 +2014,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId73"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId73"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2039,13 +2039,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId74"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId74"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2064,13 +2064,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId75"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId75"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2089,13 +2089,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId76"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId76"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2114,13 +2114,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId77"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId77"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2139,13 +2139,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId78"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId78"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2164,13 +2164,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId79"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId79"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2189,13 +2189,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId80"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId80"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2214,13 +2214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId81"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId81"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2239,13 +2239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId82"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId82"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2264,13 +2264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId83"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId83"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2289,13 +2289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId84"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId84"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2314,13 +2314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId85"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId85"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2339,13 +2339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId86"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId86"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2364,13 +2364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId87"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId87"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2389,13 +2389,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId88"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId88"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2414,13 +2414,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId89"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId89"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2439,13 +2439,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId90"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId90"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2464,13 +2464,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId91"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId91"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2489,13 +2489,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId92"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId92"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2514,13 +2514,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId93"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId93"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2539,13 +2539,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId94"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId94"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2564,13 +2564,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId95"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId95"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2589,13 +2589,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId96"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId96"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2614,13 +2614,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId97"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId97"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2639,13 +2639,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId98"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId98"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2664,13 +2664,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId99"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId99"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2689,13 +2689,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId100"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId100"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2714,13 +2714,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId101"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId101"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2739,13 +2739,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId102"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId102"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2764,13 +2764,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId103"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId103"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2789,13 +2789,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId104"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId104"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2814,13 +2814,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId105"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId105"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2839,13 +2839,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId106"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId106"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2864,13 +2864,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId107"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId107"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2889,13 +2889,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId108"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId108"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2914,13 +2914,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId109"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId109"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2939,13 +2939,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId110"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId110"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2964,13 +2964,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId111"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId111"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -2989,13 +2989,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId112"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId112"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3014,13 +3014,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId113"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId113"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3039,13 +3039,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId114"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId114"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3064,13 +3064,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId115"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId115"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3089,13 +3089,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId116"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId116"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3114,13 +3114,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId117"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId117"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3139,13 +3139,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId118"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId118"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3164,13 +3164,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId119"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId119"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3189,13 +3189,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId120"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId120"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3214,13 +3214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId121"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId121"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3239,13 +3239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId122"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId122"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3264,13 +3264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId123"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId123"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3289,13 +3289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId124"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId124"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3314,13 +3314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId125"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId125"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3339,13 +3339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId126"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId126"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3364,13 +3364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId127"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId127"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3389,13 +3389,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId128"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId128"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3414,13 +3414,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId129"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId129"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3439,13 +3439,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId130"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId130"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3464,13 +3464,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId131"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId131"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3489,13 +3489,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId132"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId132"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3514,13 +3514,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId133"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId133"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3539,13 +3539,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId134"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId134"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3564,13 +3564,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId135"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId135"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3589,13 +3589,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId136"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId136"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3614,13 +3614,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId137"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId137"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3639,13 +3639,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId138"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId138"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3664,13 +3664,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId139"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId139"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3689,13 +3689,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId140"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId140"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3714,13 +3714,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId141"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId141"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3739,13 +3739,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId142"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId142"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3764,13 +3764,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId143"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId143"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3789,13 +3789,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId144"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId144"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3814,13 +3814,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId145"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId145"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3839,13 +3839,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId146"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId146"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3864,13 +3864,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId147"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId147"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3889,13 +3889,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId148"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId148"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3914,13 +3914,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId149"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId149"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3939,13 +3939,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId150"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId150"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3964,13 +3964,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId151"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId151"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -3989,13 +3989,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId152"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId152"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4014,13 +4014,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId153"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId153"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4039,13 +4039,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId154"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId154"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4064,13 +4064,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId155"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId155"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4089,13 +4089,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId156"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId156"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4114,13 +4114,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId157"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId157"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4139,13 +4139,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId158"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId158"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4164,13 +4164,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId159"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId159"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4189,13 +4189,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId160"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId160"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4214,13 +4214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId161"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId161"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4239,13 +4239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId162"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId162"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4264,13 +4264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId163"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId163"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4289,13 +4289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId164"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId164"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4314,13 +4314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId165"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId165"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4339,13 +4339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId166"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId166"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4364,13 +4364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId167"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId167"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4389,13 +4389,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId168"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId168"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4414,13 +4414,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId169"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId169"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4439,13 +4439,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId170"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId170"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4464,13 +4464,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId171"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId171"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4489,13 +4489,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId172"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId172"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4514,13 +4514,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId173"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId173"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4539,13 +4539,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId174"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId174"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4564,13 +4564,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId175"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId175"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4589,13 +4589,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId176"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId176"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4614,13 +4614,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId177"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId177"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4639,13 +4639,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId178"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId178"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4664,13 +4664,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId179"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId179"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4689,13 +4689,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId180"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId180"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4714,13 +4714,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId181"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId181"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4739,13 +4739,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId182"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId182"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4764,13 +4764,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId183"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId183"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4789,13 +4789,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId184"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId184"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4814,13 +4814,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId185"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId185"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4839,13 +4839,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId186"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId186"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4864,13 +4864,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId187"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId187"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4889,13 +4889,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId188"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId188"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4914,13 +4914,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId189"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId189"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4939,13 +4939,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId190"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId190"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4964,13 +4964,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId191"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId191"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -4989,13 +4989,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId192"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId192"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5014,13 +5014,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId193"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId193"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5039,13 +5039,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId194"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId194"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5064,13 +5064,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId195"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId195"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5089,13 +5089,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId196"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId196"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5114,13 +5114,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId197"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId197"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5139,13 +5139,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId198"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId198"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5164,13 +5164,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId199"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId199"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5189,13 +5189,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId200"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId200"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5214,13 +5214,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId201"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId201"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5239,13 +5239,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId202"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId202"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5264,13 +5264,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId203"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId203"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5289,13 +5289,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId204"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId204"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5314,13 +5314,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId205"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId205"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5339,13 +5339,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId206"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId206"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>
@@ -5364,13 +5364,13 @@
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId207"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:blip cstate="print" r:embed="rId207"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
       </spPr>
     </pic>
     <clientData/>

</xml_diff>